<commit_message>
Fix: 7 competitor donors ARE on Collaborator (incl 3 exclusive); add Collaborator prices
</commit_message>
<xml_diff>
--- a/1kredit-donors-buy-list.xlsx
+++ b/1kredit-donors-buy-list.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Доноры конкурентов" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Доноры конкурентов'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Доноры конкурентов'!$A$1:$J$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,18 +452,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,7 +475,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ссылается на (конкурент)</t>
+          <t>Ссылается на</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -494,20 +495,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ИКС (Miralinks)</t>
+          <t>GoGetLinks ₽</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>GoGetLinks ₽ (статья)</t>
+          <t>Collaborator $</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Где купить</t>
+          <t>Collaborator ₽≈</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Где дешевле</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Лучшая цена ₽</t>
         </is>
@@ -536,17 +542,16 @@
         <v>159</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="G2" s="2" t="n">
         <v>567</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="J2" s="2" t="n">
         <v>159</v>
       </c>
     </row>
@@ -573,17 +578,16 @@
         <v>204</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="G3" s="2" t="n">
         <v>442</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="J3" s="2" t="n">
         <v>204</v>
       </c>
     </row>
@@ -609,16 +613,15 @@
       <c r="E4" s="2" t="n">
         <v>238</v>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>50</v>
-      </c>
+      <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="J4" s="2" t="n">
         <v>238</v>
       </c>
     </row>
@@ -645,29 +648,28 @@
         <v>280</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" s="2" t="n">
         <v>743</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="J5" s="2" t="n">
         <v>280</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>vd-tv.ru</t>
+          <t>sveto-copy.com</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>tascredit / avto-dengi</t>
+          <t>avto-dengi</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -676,35 +678,38 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>160</v>
-      </c>
       <c r="G6" s="2" t="n">
-        <v>1429</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Miralinks</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>500</v>
+        <v>3.6</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>281</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>281</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>sveto-copy.com</t>
+          <t>vd-tv.ru</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>avto-dengi</t>
+          <t>tascredit / avto-dengi</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -713,23 +718,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>170</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>GoGetLinks</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n">
+        <v>1429</v>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Miralinks</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
         <v>500</v>
       </c>
     </row>
@@ -755,16 +759,15 @@
       <c r="E8" s="2" t="n">
         <v>588</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>20</v>
-      </c>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>588</v>
       </c>
     </row>
@@ -790,16 +793,15 @@
       <c r="E9" s="2" t="n">
         <v>599</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>50</v>
-      </c>
+      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>599</v>
       </c>
     </row>
@@ -820,22 +822,25 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>705</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Miralinks</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>705</v>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>702</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>702</v>
       </c>
     </row>
     <row r="11">
@@ -861,17 +866,16 @@
         <v>845</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G11" s="2" t="n">
         <v>1136</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="J11" s="2" t="n">
         <v>845</v>
       </c>
     </row>
@@ -898,319 +902,341 @@
         <v>1499</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="G12" s="2" t="n">
         <v>1428</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>GoGetLinks</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="J12" s="2" t="n">
         <v>1428</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>wfin.kz</t>
+          <t>churchill.kz</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>bcc (mortgage)</t>
+          <t>solva</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Недвижимость</t>
+          <t>Залог авто</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>7900</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Miralinks</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>7900</v>
+        <v>46</v>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>3510</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>3510</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ustinka.kz</t>
+          <t>wfin.kz</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>solva /pod-zalog-auto</t>
+          <t>bcc (mortgage)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Залог авто</t>
+          <t>Недвижимость</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>14500</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>460</v>
-      </c>
+        <v>7900</v>
+      </c>
+      <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
-        <v>14500</v>
+      <c r="J14" s="2" t="n">
+        <v>7900</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>upl.uz</t>
+          <t>ustinka.kz</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>solva /business</t>
+          <t>solva /pod-zalog-auto</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Кредит для ИП</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n"/>
+          <t>Залог авто</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>41</v>
+      </c>
       <c r="E15" s="2" t="n">
-        <v>33000</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>1930</v>
-      </c>
+        <v>14500</v>
+      </c>
+      <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n">
-        <v>33000</v>
+      <c r="J15" s="2" t="n">
+        <v>14500</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>astanatv.kz</t>
+          <t>kstnews.kz</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>bcc (ИП)</t>
+          <t>berekebank</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Кредит для ИП</t>
+          <t>Недвижимость</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>45000</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>510</v>
-      </c>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Miralinks</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>45000</v>
+        <v>46</v>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>23400</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>23400</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>mail.kz</t>
+          <t>kn.kz</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>solva /business</t>
+          <t>solva</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Кредит для ИП</t>
+          <t>Залог авто</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>153512</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>2090</v>
-      </c>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Miralinks</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="n">
-        <v>153512</v>
+        <v>40</v>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n">
+        <v>355</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>27690</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>27690</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>upl.uz</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>solva /business</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Кредит для ИП</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n">
+        <v>33000</v>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Miralinks</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>astanatv.kz</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>bcc (ИП)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Кредит для ИП</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n">
+        <v>424</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>33072</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>33072</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>profit.kz</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>solva /business</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Кредит для ИП</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D20" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>187848</v>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n">
+        <v>687</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>53586</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Collaborator</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>53586</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>mail.kz</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>solva /business</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Кредит для ИП</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="E18" s="2" t="n">
-        <v>187848</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>410</v>
-      </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="E21" s="2" t="n">
+        <v>153512</v>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Miralinks</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>187848</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>kstnews.kz</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>berekebank</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Недвижимость</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Аутрич / нет на биржах</t>
-        </is>
-      </c>
-      <c r="I19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>kn.kz</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>solva</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Залог авто</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Аутрич / нет на биржах</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>nacredit.kz</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>halyk (рефинанс)</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Рефинансирование</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Аутрич / нет на биржах</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="2" t="n">
+        <v>153512</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>gdezaim.kz</t>
+          <t>nacredit.kz</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1224,32 +1250,33 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>profinance.kz</t>
+          <t>gdezaim.kz</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>forte / kmf / halyk</t>
+          <t>halyk (рефинанс)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Мульти-кластер</t>
+          <t>Рефинансирование</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1258,41 +1285,43 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>churchill.kz</t>
+          <t>profinance.kz</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>solva</t>
+          <t>forte / kmf / halyk</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Залог авто</t>
+          <t>Мульти-кластер</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1316,12 +1345,13 @@
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1345,12 +1375,13 @@
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1374,12 +1405,13 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1403,17 +1435,18 @@
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Аутрич / нет на биржах</t>
         </is>
       </c>
-      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>ИТОГО купить все доступные (17 шт.), ₽</t>
+          <t>ИТОГО доступных (20), ₽</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1423,12 +1456,13 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" s="4" t="n">
-        <v>447806</v>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" s="4" t="n">
+        <v>355994</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:J28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>